<commit_message>
Update LubaNur database after transaction
</commit_message>
<xml_diff>
--- a/system_database.xlsx
+++ b/system_database.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Stock" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Expenses" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Cargo_Companies" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Stock_Movements" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Product_Costs" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -6047,7 +6047,7 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>مدفوع بالكامل</t>
+          <t>قيد التحصيل</t>
         </is>
       </c>
       <c r="P77" t="n">
@@ -11339,43 +11339,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>DateTime</t>
+          <t>Item_Name</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Item_Name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Operation</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Quantity</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Before_Qty</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>After_Qty</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Note</t>
+          <t>Unit_Cost</t>
         </is>
       </c>
     </row>

</xml_diff>